<commit_message>
trabajo y revision de los modulos principales de importacion, producccion, ventas
</commit_message>
<xml_diff>
--- a/bin/Debug/net8.0-windows10.0.19041/RollosCortados.xlsx
+++ b/bin/Debug/net8.0-windows10.0.19041/RollosCortados.xlsx
@@ -70,160 +70,166 @@
     <x:t>Numero</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">06758                                             </x:t>
+    <x:t xml:space="preserve">06758                    </x:t>
   </x:si>
   <x:si>
     <x:t>TOP TRANSFER AP904 SK60</x:t>
   </x:si>
   <x:si>
-    <x:t>RC30641</x:t>
+    <x:t>RC30689</x:t>
   </x:si>
   <x:si>
     <x:t>42805211</x:t>
   </x:si>
   <x:si>
-    <x:t>n/t</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30642</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30643</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30644</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30645</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30646</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30647</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30648</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30649</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30650</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30651</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30652</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30653</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30654</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30655</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30656</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30657</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30658</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30659</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30660</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30661</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30662</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30663</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30664</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30665</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30666</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30667</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30668</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30669</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30670</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30671</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30672</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30673</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30674</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30675</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30676</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30677</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30678</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30679</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30680</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30681</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30682</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30683</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30684</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30685</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30686</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30687</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30688</x:t>
+    <x:t>n/a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30690</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30691</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30692</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30693</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30694</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30695</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30696</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30697</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30698</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30699</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30700</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30701</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30702</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30703</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30704</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30705</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30706</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30707</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30708</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30709</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30710</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30711</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30712</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30713</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30714</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30715</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30716</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30717</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30718</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30719</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30720</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30721</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30722</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30723</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30724</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30725</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30726</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30727</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30728</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30729</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30730</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30731</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30732</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30733</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30734</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30735</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30736</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -593,7 +599,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11.424911" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="26.424911" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15.139196" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="25.139196" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.282054" style="0" customWidth="1"/>
@@ -696,17 +702,23 @@
       <x:c r="I2" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J2" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M2" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N2" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O2" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P2" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q2" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R2" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:18">
@@ -720,7 +732,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>2</x:v>
@@ -737,17 +749,23 @@
       <x:c r="I3" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J3" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M3" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N3" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O3" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P3" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q3" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R3" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:18">
@@ -761,7 +779,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>5</x:v>
@@ -778,17 +796,23 @@
       <x:c r="I4" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J4" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M4" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N4" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O4" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P4" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q4" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R4" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:18">
@@ -802,7 +826,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E5" s="0">
         <x:v>3</x:v>
@@ -819,17 +843,23 @@
       <x:c r="I5" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J5" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M5" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N5" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O5" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P5" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q5" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R5" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:18">
@@ -843,7 +873,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E6" s="0">
         <x:v>2</x:v>
@@ -860,17 +890,23 @@
       <x:c r="I6" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J6" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M6" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N6" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O6" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P6" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q6" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R6" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:18">
@@ -884,7 +920,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E7" s="0">
         <x:v>2</x:v>
@@ -901,17 +937,23 @@
       <x:c r="I7" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J7" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M7" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N7" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O7" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P7" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q7" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R7" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:18">
@@ -925,7 +967,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E8" s="0">
         <x:v>5</x:v>
@@ -942,17 +984,23 @@
       <x:c r="I8" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J8" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M8" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N8" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O8" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P8" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q8" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R8" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:18">
@@ -966,7 +1014,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E9" s="0">
         <x:v>3</x:v>
@@ -983,17 +1031,23 @@
       <x:c r="I9" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J9" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M9" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N9" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O9" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P9" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q9" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R9" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:18">
@@ -1007,7 +1061,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E10" s="0">
         <x:v>2</x:v>
@@ -1024,17 +1078,23 @@
       <x:c r="I10" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J10" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M10" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N10" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O10" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P10" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q10" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R10" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:18">
@@ -1048,7 +1108,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E11" s="0">
         <x:v>2</x:v>
@@ -1065,17 +1125,23 @@
       <x:c r="I11" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J11" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M11" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N11" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O11" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P11" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q11" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R11" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:18">
@@ -1089,7 +1155,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E12" s="0">
         <x:v>5</x:v>
@@ -1106,17 +1172,23 @@
       <x:c r="I12" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J12" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M12" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N12" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O12" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P12" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q12" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R12" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:18">
@@ -1130,7 +1202,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E13" s="0">
         <x:v>3</x:v>
@@ -1147,17 +1219,23 @@
       <x:c r="I13" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J13" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M13" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N13" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O13" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P13" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q13" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R13" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:18">
@@ -1171,7 +1249,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E14" s="0">
         <x:v>2</x:v>
@@ -1188,17 +1266,23 @@
       <x:c r="I14" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J14" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M14" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N14" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O14" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P14" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q14" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R14" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:18">
@@ -1212,7 +1296,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E15" s="0">
         <x:v>2</x:v>
@@ -1229,17 +1313,23 @@
       <x:c r="I15" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J15" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M15" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N15" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O15" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P15" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q15" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R15" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:18">
@@ -1253,7 +1343,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E16" s="0">
         <x:v>5</x:v>
@@ -1270,17 +1360,23 @@
       <x:c r="I16" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J16" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M16" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N16" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O16" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P16" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q16" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R16" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:18">
@@ -1294,7 +1390,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E17" s="0">
         <x:v>3</x:v>
@@ -1311,17 +1407,23 @@
       <x:c r="I17" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J17" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M17" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N17" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O17" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P17" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q17" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R17" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:18">
@@ -1335,7 +1437,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E18" s="0">
         <x:v>2</x:v>
@@ -1352,17 +1454,23 @@
       <x:c r="I18" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J18" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M18" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N18" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O18" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P18" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q18" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R18" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:18">
@@ -1376,7 +1484,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E19" s="0">
         <x:v>2</x:v>
@@ -1393,17 +1501,23 @@
       <x:c r="I19" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J19" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M19" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N19" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O19" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P19" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q19" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R19" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:18">
@@ -1417,7 +1531,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E20" s="0">
         <x:v>5</x:v>
@@ -1434,17 +1548,23 @@
       <x:c r="I20" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J20" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M20" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N20" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O20" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P20" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q20" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R20" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:18">
@@ -1458,7 +1578,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E21" s="0">
         <x:v>3</x:v>
@@ -1475,17 +1595,23 @@
       <x:c r="I21" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J21" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M21" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N21" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O21" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P21" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q21" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R21" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:18">
@@ -1499,7 +1625,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E22" s="0">
         <x:v>2</x:v>
@@ -1516,17 +1642,23 @@
       <x:c r="I22" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J22" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M22" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N22" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O22" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P22" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q22" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R22" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:18">
@@ -1540,7 +1672,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E23" s="0">
         <x:v>2</x:v>
@@ -1557,17 +1689,23 @@
       <x:c r="I23" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J23" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M23" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N23" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O23" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P23" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q23" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R23" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:18">
@@ -1581,7 +1719,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E24" s="0">
         <x:v>5</x:v>
@@ -1598,17 +1736,23 @@
       <x:c r="I24" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J24" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M24" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N24" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O24" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P24" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q24" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R24" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:18">
@@ -1622,7 +1766,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E25" s="0">
         <x:v>3</x:v>
@@ -1639,17 +1783,23 @@
       <x:c r="I25" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J25" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M25" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N25" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O25" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P25" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q25" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R25" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:18">
@@ -1663,7 +1813,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="E26" s="0">
         <x:v>2</x:v>
@@ -1680,17 +1830,23 @@
       <x:c r="I26" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J26" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M26" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N26" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O26" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P26" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q26" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R26" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:18">
@@ -1704,7 +1860,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E27" s="0">
         <x:v>2</x:v>
@@ -1721,17 +1877,23 @@
       <x:c r="I27" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J27" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M27" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N27" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O27" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P27" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q27" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R27" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:18">
@@ -1745,7 +1907,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E28" s="0">
         <x:v>5</x:v>
@@ -1762,17 +1924,23 @@
       <x:c r="I28" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J28" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M28" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N28" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O28" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P28" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q28" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R28" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:18">
@@ -1786,7 +1954,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E29" s="0">
         <x:v>3</x:v>
@@ -1803,17 +1971,23 @@
       <x:c r="I29" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J29" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M29" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N29" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O29" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P29" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q29" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R29" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:18">
@@ -1827,7 +2001,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E30" s="0">
         <x:v>2</x:v>
@@ -1844,17 +2018,23 @@
       <x:c r="I30" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J30" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M30" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N30" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O30" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P30" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q30" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R30" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:18">
@@ -1868,7 +2048,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E31" s="0">
         <x:v>2</x:v>
@@ -1885,17 +2065,23 @@
       <x:c r="I31" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J31" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M31" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N31" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O31" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P31" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q31" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R31" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:18">
@@ -1909,7 +2095,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="E32" s="0">
         <x:v>5</x:v>
@@ -1926,17 +2112,23 @@
       <x:c r="I32" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J32" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M32" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N32" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O32" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P32" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q32" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R32" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:18">
@@ -1950,7 +2142,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="E33" s="0">
         <x:v>3</x:v>
@@ -1967,17 +2159,23 @@
       <x:c r="I33" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J33" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M33" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N33" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O33" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P33" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q33" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R33" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:18">
@@ -1991,7 +2189,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E34" s="0">
         <x:v>2</x:v>
@@ -2008,17 +2206,23 @@
       <x:c r="I34" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J34" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M34" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N34" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O34" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P34" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q34" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R34" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:18">
@@ -2032,7 +2236,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E35" s="0">
         <x:v>2</x:v>
@@ -2049,17 +2253,23 @@
       <x:c r="I35" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J35" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M35" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N35" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O35" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P35" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q35" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R35" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:18">
@@ -2073,7 +2283,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E36" s="0">
         <x:v>5</x:v>
@@ -2090,17 +2300,23 @@
       <x:c r="I36" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J36" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M36" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N36" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O36" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P36" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q36" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R36" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:18">
@@ -2114,7 +2330,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E37" s="0">
         <x:v>3</x:v>
@@ -2131,17 +2347,23 @@
       <x:c r="I37" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J37" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M37" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N37" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O37" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P37" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q37" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R37" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:18">
@@ -2155,7 +2377,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D38" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E38" s="0">
         <x:v>2</x:v>
@@ -2172,17 +2394,23 @@
       <x:c r="I38" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J38" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M38" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N38" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O38" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P38" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q38" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R38" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:18">
@@ -2196,7 +2424,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D39" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E39" s="0">
         <x:v>2</x:v>
@@ -2213,17 +2441,23 @@
       <x:c r="I39" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J39" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M39" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N39" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O39" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P39" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q39" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R39" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:18">
@@ -2237,7 +2471,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D40" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="E40" s="0">
         <x:v>5</x:v>
@@ -2254,17 +2488,23 @@
       <x:c r="I40" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J40" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M40" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N40" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O40" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P40" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q40" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R40" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:18">
@@ -2278,7 +2518,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D41" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E41" s="0">
         <x:v>3</x:v>
@@ -2295,17 +2535,23 @@
       <x:c r="I41" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J41" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M41" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N41" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O41" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P41" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q41" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R41" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:18">
@@ -2319,7 +2565,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D42" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E42" s="0">
         <x:v>2</x:v>
@@ -2336,17 +2582,23 @@
       <x:c r="I42" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J42" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M42" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N42" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O42" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P42" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q42" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R42" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:18">
@@ -2360,7 +2612,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D43" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E43" s="0">
         <x:v>2</x:v>
@@ -2377,17 +2629,23 @@
       <x:c r="I43" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J43" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M43" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N43" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O43" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P43" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q43" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R43" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:18">
@@ -2401,7 +2659,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D44" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E44" s="0">
         <x:v>5</x:v>
@@ -2418,17 +2676,23 @@
       <x:c r="I44" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J44" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M44" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N44" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O44" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P44" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q44" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R44" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:18">
@@ -2442,7 +2706,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D45" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="E45" s="0">
         <x:v>3</x:v>
@@ -2459,17 +2723,23 @@
       <x:c r="I45" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J45" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M45" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N45" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O45" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P45" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q45" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R45" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:18">
@@ -2483,7 +2753,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D46" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E46" s="0">
         <x:v>2</x:v>
@@ -2500,17 +2770,23 @@
       <x:c r="I46" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J46" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M46" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N46" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O46" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P46" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q46" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R46" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:18">
@@ -2524,7 +2800,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D47" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E47" s="0">
         <x:v>2</x:v>
@@ -2541,17 +2817,23 @@
       <x:c r="I47" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J47" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M47" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N47" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O47" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P47" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q47" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R47" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:18">
@@ -2565,7 +2847,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D48" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E48" s="0">
         <x:v>5</x:v>
@@ -2582,17 +2864,23 @@
       <x:c r="I48" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J48" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M48" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N48" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O48" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P48" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q48" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R48" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:18">
@@ -2606,7 +2894,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D49" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E49" s="0">
         <x:v>3</x:v>
@@ -2623,17 +2911,23 @@
       <x:c r="I49" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J49" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="M49" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N49" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O49" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P49" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="Q49" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R49" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
trabajo con el formulario de productos
</commit_message>
<xml_diff>
--- a/bin/Debug/net8.0-windows10.0.19041/RollosCortados.xlsx
+++ b/bin/Debug/net8.0-windows10.0.19041/RollosCortados.xlsx
@@ -70,13 +70,13 @@
     <x:t>Numero</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">06758                    </x:t>
+    <x:t xml:space="preserve">06758                                                                                               </x:t>
   </x:si>
   <x:si>
     <x:t>TOP TRANSFER AP904 SK60</x:t>
   </x:si>
   <x:si>
-    <x:t>RC30689</x:t>
+    <x:t>RC30737</x:t>
   </x:si>
   <x:si>
     <x:t>42805211</x:t>
@@ -88,148 +88,103 @@
     <x:t>0</x:t>
   </x:si>
   <x:si>
-    <x:t>8</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30690</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30691</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30692</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30693</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30694</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30695</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30696</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30697</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30698</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30699</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30700</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30701</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30702</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30703</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30704</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30705</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30706</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30707</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30708</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30709</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30710</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30711</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30712</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30713</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30714</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30715</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30716</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30717</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30718</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30719</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30720</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30721</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30722</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30723</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30724</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30725</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30726</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30727</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30728</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30729</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30730</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30731</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30732</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30733</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30734</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30735</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30736</x:t>
+    <x:t>14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30738</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30739</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30740</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30741</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30742</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30743</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30744</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30745</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30746</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30747</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30748</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30749</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30750</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30751</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30752</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30753</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30754</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30755</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30756</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30757</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30758</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30759</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30760</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30761</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30762</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30763</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30764</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30765</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30766</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30767</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30768</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30769</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -595,11 +550,11 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:R49"/>
+  <x:dimension ref="A1:R34"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11.424911" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15.139196" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="49.282054" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="25.139196" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.282054" style="0" customWidth="1"/>
@@ -688,13 +643,13 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H2" s="0">
         <x:v>0</x:v>
@@ -735,13 +690,13 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H3" s="0">
         <x:v>0</x:v>
@@ -782,13 +737,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>96</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H4" s="0">
         <x:v>0</x:v>
@@ -829,13 +784,13 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>57.6</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H5" s="0">
         <x:v>0</x:v>
@@ -876,13 +831,13 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H6" s="0">
         <x:v>0</x:v>
@@ -923,13 +878,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H7" s="0">
         <x:v>0</x:v>
@@ -970,13 +925,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>96</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H8" s="0">
         <x:v>0</x:v>
@@ -1017,13 +972,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>57.6</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H9" s="0">
         <x:v>0</x:v>
@@ -1064,13 +1019,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H10" s="0">
         <x:v>0</x:v>
@@ -1111,13 +1066,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H11" s="0">
         <x:v>0</x:v>
@@ -1158,13 +1113,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>96</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H12" s="0">
         <x:v>0</x:v>
@@ -1205,13 +1160,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>57.6</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H13" s="0">
         <x:v>0</x:v>
@@ -1252,13 +1207,13 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H14" s="0">
         <x:v>0</x:v>
@@ -1299,13 +1254,13 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H15" s="0">
         <x:v>0</x:v>
@@ -1346,13 +1301,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>96</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H16" s="0">
         <x:v>0</x:v>
@@ -1393,13 +1348,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>57.6</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H17" s="0">
         <x:v>0</x:v>
@@ -1440,13 +1395,13 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H18" s="0">
         <x:v>0</x:v>
@@ -1487,13 +1442,13 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H19" s="0">
         <x:v>0</x:v>
@@ -1534,13 +1489,13 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>96</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H20" s="0">
         <x:v>0</x:v>
@@ -1581,13 +1536,13 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>57.6</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H21" s="0">
         <x:v>0</x:v>
@@ -1628,13 +1583,13 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="E22" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H22" s="0">
         <x:v>0</x:v>
@@ -1675,13 +1630,13 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H23" s="0">
         <x:v>0</x:v>
@@ -1722,13 +1677,13 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>96</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H24" s="0">
         <x:v>0</x:v>
@@ -1769,13 +1724,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>57.6</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H25" s="0">
         <x:v>0</x:v>
@@ -1816,13 +1771,13 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H26" s="0">
         <x:v>0</x:v>
@@ -1863,13 +1818,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="E27" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H27" s="0">
         <x:v>0</x:v>
@@ -1910,13 +1865,13 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>96</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H28" s="0">
         <x:v>0</x:v>
@@ -1957,13 +1912,13 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="E29" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F29" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G29" s="0">
-        <x:v>57.6</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H29" s="0">
         <x:v>0</x:v>
@@ -2004,13 +1959,13 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="E30" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F30" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G30" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H30" s="0">
         <x:v>0</x:v>
@@ -2051,13 +2006,13 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="E31" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F31" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G31" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H31" s="0">
         <x:v>0</x:v>
@@ -2098,13 +2053,13 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="E32" s="0">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F32" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G32" s="0">
-        <x:v>96</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H32" s="0">
         <x:v>0</x:v>
@@ -2145,13 +2100,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="E33" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F33" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G33" s="0">
-        <x:v>57.6</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H33" s="0">
         <x:v>0</x:v>
@@ -2192,13 +2147,13 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="E34" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F34" s="0">
-        <x:v>1600</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G34" s="0">
-        <x:v>38.4</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H34" s="0">
         <x:v>0</x:v>
@@ -2222,711 +2177,6 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="R34" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" spans="1:18">
-      <x:c r="A35" s="0">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="B35" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C35" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D35" s="0" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="E35" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F35" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G35" s="0">
-        <x:v>38.4</x:v>
-      </x:c>
-      <x:c r="H35" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I35" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M35" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N35" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O35" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P35" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q35" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R35" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" spans="1:18">
-      <x:c r="A36" s="0">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B36" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C36" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D36" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="E36" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F36" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G36" s="0">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="H36" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I36" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M36" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N36" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O36" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P36" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q36" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R36" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" spans="1:18">
-      <x:c r="A37" s="0">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B37" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C37" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D37" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="E37" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F37" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G37" s="0">
-        <x:v>57.6</x:v>
-      </x:c>
-      <x:c r="H37" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I37" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M37" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N37" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O37" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P37" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q37" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R37" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" spans="1:18">
-      <x:c r="A38" s="0">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B38" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C38" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D38" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="E38" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F38" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G38" s="0">
-        <x:v>38.4</x:v>
-      </x:c>
-      <x:c r="H38" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I38" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M38" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N38" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O38" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P38" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q38" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R38" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" spans="1:18">
-      <x:c r="A39" s="0">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B39" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C39" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D39" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="E39" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F39" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G39" s="0">
-        <x:v>38.4</x:v>
-      </x:c>
-      <x:c r="H39" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I39" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M39" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N39" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O39" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P39" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q39" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R39" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" spans="1:18">
-      <x:c r="A40" s="0">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B40" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C40" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D40" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="E40" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F40" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G40" s="0">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="H40" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I40" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M40" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N40" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O40" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P40" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q40" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R40" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" spans="1:18">
-      <x:c r="A41" s="0">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="B41" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C41" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D41" s="0" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="E41" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F41" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G41" s="0">
-        <x:v>57.6</x:v>
-      </x:c>
-      <x:c r="H41" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I41" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M41" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N41" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O41" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P41" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q41" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R41" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" spans="1:18">
-      <x:c r="A42" s="0">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B42" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C42" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D42" s="0" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="E42" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F42" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G42" s="0">
-        <x:v>38.4</x:v>
-      </x:c>
-      <x:c r="H42" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I42" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M42" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N42" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O42" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P42" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q42" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R42" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" spans="1:18">
-      <x:c r="A43" s="0">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B43" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C43" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D43" s="0" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="E43" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F43" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G43" s="0">
-        <x:v>38.4</x:v>
-      </x:c>
-      <x:c r="H43" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I43" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M43" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N43" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O43" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P43" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q43" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R43" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" spans="1:18">
-      <x:c r="A44" s="0">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="B44" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C44" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D44" s="0" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="E44" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F44" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G44" s="0">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="H44" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I44" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M44" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N44" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O44" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P44" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q44" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R44" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" spans="1:18">
-      <x:c r="A45" s="0">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="B45" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C45" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D45" s="0" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="E45" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F45" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G45" s="0">
-        <x:v>57.6</x:v>
-      </x:c>
-      <x:c r="H45" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I45" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M45" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N45" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O45" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P45" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q45" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R45" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" spans="1:18">
-      <x:c r="A46" s="0">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="B46" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C46" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D46" s="0" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="E46" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F46" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G46" s="0">
-        <x:v>38.4</x:v>
-      </x:c>
-      <x:c r="H46" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I46" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M46" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N46" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O46" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P46" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q46" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R46" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" spans="1:18">
-      <x:c r="A47" s="0">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="B47" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C47" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D47" s="0" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="E47" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F47" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G47" s="0">
-        <x:v>38.4</x:v>
-      </x:c>
-      <x:c r="H47" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I47" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M47" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N47" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O47" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P47" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q47" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R47" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" spans="1:18">
-      <x:c r="A48" s="0">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B48" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C48" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D48" s="0" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="E48" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F48" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G48" s="0">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="H48" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I48" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M48" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N48" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O48" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P48" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q48" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R48" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" spans="1:18">
-      <x:c r="A49" s="0">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="B49" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C49" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D49" s="0" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="E49" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F49" s="0">
-        <x:v>1600</x:v>
-      </x:c>
-      <x:c r="G49" s="0">
-        <x:v>57.6</x:v>
-      </x:c>
-      <x:c r="H49" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I49" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M49" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N49" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O49" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="P49" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="Q49" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R49" s="0" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
trabajo en la conexion al servidor local y produccion con el manejo de ambiente en el appsettings
</commit_message>
<xml_diff>
--- a/bin/Debug/net8.0-windows10.0.19041/RollosCortados.xlsx
+++ b/bin/Debug/net8.0-windows10.0.19041/RollosCortados.xlsx
@@ -70,7 +70,7 @@
     <x:t>Numero</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">06758                                                                                               </x:t>
+    <x:t xml:space="preserve">06758                    </x:t>
   </x:si>
   <x:si>
     <x:t>TOP TRANSFER AP904 SK60</x:t>
@@ -88,7 +88,7 @@
     <x:t>0</x:t>
   </x:si>
   <x:si>
-    <x:t>14</x:t>
+    <x:t>16</x:t>
   </x:si>
   <x:si>
     <x:t>RC30738</x:t>
@@ -554,7 +554,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11.424911" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="49.282054" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15.139196" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="25.139196" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.282054" style="0" customWidth="1"/>

</xml_diff>